<commit_message>
Correct minor error in docs
</commit_message>
<xml_diff>
--- a/data/TestData.xlsx
+++ b/data/TestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ee85442dac9ca7a7/Documents/Julia/ExcelFiles/ExcelFiles.jl/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C77CE8C6-941C-4A2C-841B-13651ABB1B0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="8_{C77CE8C6-941C-4A2C-841B-13651ABB1B0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{93DAB118-4432-439F-A2CD-6A7A4126E8E8}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{67B4354B-AE01-4157-BE47-00198EBFE8E7}"/>
   </bookViews>
@@ -121,7 +121,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="172" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -156,7 +156,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">

</xml_diff>